<commit_message>
sawabt icon and exitfullscreen
</commit_message>
<xml_diff>
--- a/li.xlsx
+++ b/li.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\power bi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69FF6CD0-EB30-4CB3-A20C-8AAA6923BFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B005AF-28BA-4EC5-B32A-95197A5DA7F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="705" activeTab="8" xr2:uid="{12120B74-1E2A-4740-BDBD-5E619114E9BB}"/>
   </bookViews>
@@ -150,7 +150,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="84">
   <si>
     <t>tradeid</t>
   </si>
@@ -390,9 +390,6 @@
   </si>
   <si>
     <t>Jan</t>
-  </si>
-  <si>
-    <t>Feb</t>
   </si>
   <si>
     <t>hamid taha</t>
@@ -1832,9 +1829,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'pivot table sales'!$D$5:$D$9</c:f>
+              <c:f>'pivot table sales'!$D$5:$D$10</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>Ahmed Said</c:v>
                 </c:pt>
@@ -1842,9 +1839,12 @@
                   <c:v>Ali Ramadan</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>Fathy Ali</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>Khaled Hassan</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>Tamer Mohamed</c:v>
                 </c:pt>
               </c:strCache>
@@ -1852,21 +1852,24 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'pivot table sales'!$E$5:$E$9</c:f>
+              <c:f>'pivot table sales'!$E$5:$E$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>1140</c:v>
+                  <c:v>900</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>760</c:v>
+                  <c:v>2400</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1140</c:v>
+                  <c:v>1500</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>190</c:v>
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2100</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2282,13 +2285,13 @@
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Khaled Hassan</c:v>
+                  <c:v>Tamer Mohamed</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Ali Ramadan</c:v>
+                  <c:v>Fathy Ali</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Ahmed Said</c:v>
+                  <c:v>Ali Ramadan</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2300,13 +2303,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>1140</c:v>
+                  <c:v>2100</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>760</c:v>
+                  <c:v>1500</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1140</c:v>
+                  <c:v>2400</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2714,71 +2717,23 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'pivot table sales'!$A$5:$A$14</c:f>
+              <c:f>'pivot table sales'!$A$5:$A$6</c:f>
               <c:strCache>
-                <c:ptCount val="9"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Headset</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Keyboard</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Laptop</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Monitor</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Mouse</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Printer</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Scanner</c:v>
-                </c:pt>
-                <c:pt idx="7">
                   <c:v>Speaker</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>gamer</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'pivot table sales'!$B$5:$B$14</c:f>
+              <c:f>'pivot table sales'!$B$5:$B$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="9"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>3600</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>3230</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>306000</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>12000</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>4200</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>79800</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>10500</c:v>
-                </c:pt>
-                <c:pt idx="7">
                   <c:v>7200</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>168</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3187,35 +3142,23 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'pivot table sales'!$A$36:$A$39</c:f>
+              <c:f>'pivot table sales'!$A$36:$A$37</c:f>
               <c:strCache>
-                <c:ptCount val="3"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Laptop</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Printer</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Monitor</c:v>
+                  <c:v>Speaker</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'pivot table sales'!$B$36:$B$39</c:f>
+              <c:f>'pivot table sales'!$B$36:$B$37</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>306000</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>79800</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>12000</c:v>
+                  <c:v>7200</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3636,29 +3579,23 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'pivot table sales'!$H$5:$H$7</c:f>
+              <c:f>'pivot table sales'!$H$5:$H$6</c:f>
               <c:strCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>Jan</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Feb</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'pivot table sales'!$I$5:$I$7</c:f>
+              <c:f>'pivot table sales'!$I$5:$I$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>2850</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>380</c:v>
+                  <c:v>7200</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4109,71 +4046,23 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'pivot table sales'!$A$5:$A$14</c:f>
+              <c:f>'pivot table sales'!$A$5:$A$6</c:f>
               <c:strCache>
-                <c:ptCount val="9"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Headset</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Keyboard</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Laptop</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Monitor</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Mouse</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Printer</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Scanner</c:v>
-                </c:pt>
-                <c:pt idx="7">
                   <c:v>Speaker</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>gamer</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'pivot table sales'!$B$5:$B$14</c:f>
+              <c:f>'pivot table sales'!$B$5:$B$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="9"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>3600</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>3230</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>306000</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>12000</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>4200</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>79800</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>10500</c:v>
-                </c:pt>
-                <c:pt idx="7">
                   <c:v>7200</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>168</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4447,13 +4336,13 @@
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Khaled Hassan</c:v>
+                  <c:v>Tamer Mohamed</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Ali Ramadan</c:v>
+                  <c:v>Fathy Ali</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Ahmed Said</c:v>
+                  <c:v>Ali Ramadan</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -4465,13 +4354,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>1140</c:v>
+                  <c:v>2100</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>760</c:v>
+                  <c:v>1500</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1140</c:v>
+                  <c:v>2400</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4761,71 +4650,23 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'pivot table sales'!$A$5:$A$14</c:f>
+              <c:f>'pivot table sales'!$A$5:$A$6</c:f>
               <c:strCache>
-                <c:ptCount val="9"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Headset</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Keyboard</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Laptop</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Monitor</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Mouse</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Printer</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Scanner</c:v>
-                </c:pt>
-                <c:pt idx="7">
                   <c:v>Speaker</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>gamer</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'pivot table sales'!$B$5:$B$14</c:f>
+              <c:f>'pivot table sales'!$B$5:$B$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="9"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>3600</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>3230</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>306000</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>12000</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>4200</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>79800</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>10500</c:v>
-                </c:pt>
-                <c:pt idx="7">
                   <c:v>7200</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>168</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5116,35 +4957,23 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'pivot table sales'!$A$36:$A$39</c:f>
+              <c:f>'pivot table sales'!$A$36:$A$37</c:f>
               <c:strCache>
-                <c:ptCount val="3"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Laptop</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Printer</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Monitor</c:v>
+                  <c:v>Speaker</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'pivot table sales'!$B$36:$B$39</c:f>
+              <c:f>'pivot table sales'!$B$36:$B$37</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>306000</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>79800</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>12000</c:v>
+                  <c:v>7200</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10952,7 +10781,7 @@
                 <a:latin typeface="Aptos Narrow"/>
               </a:rPr>
               <a:pPr/>
-              <a:t>3230</a:t>
+              <a:t>7200</a:t>
             </a:fld>
             <a:endParaRPr lang="en-US" sz="2000" b="1">
               <a:solidFill>
@@ -11189,7 +11018,7 @@
               <a:latin typeface="Aptos Narrow"/>
             </a:rPr>
             <a:pPr/>
-            <a:t>646</a:t>
+            <a:t>900</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="2000" b="1">
             <a:solidFill>
@@ -11425,7 +11254,7 @@
               <a:latin typeface="Aptos Narrow"/>
             </a:rPr>
             <a:pPr/>
-            <a:t>5</a:t>
+            <a:t>8</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="2000" b="1">
             <a:solidFill>
@@ -11661,7 +11490,7 @@
               <a:latin typeface="Aptos Narrow"/>
             </a:rPr>
             <a:pPr/>
-            <a:t>1140</a:t>
+            <a:t>2100</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="2000" b="1">
             <a:solidFill>
@@ -11934,7 +11763,7 @@
               <a:latin typeface="Aptos Narrow"/>
             </a:rPr>
             <a:pPr/>
-            <a:t>190</a:t>
+            <a:t>300</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="2000" b="1">
             <a:solidFill>
@@ -13063,7 +12892,7 @@
                 <a:latin typeface="Aptos Narrow"/>
               </a:rPr>
               <a:pPr/>
-              <a:t>3230</a:t>
+              <a:t>7200</a:t>
             </a:fld>
             <a:endParaRPr lang="en-US" sz="2000" b="1">
               <a:solidFill>
@@ -13300,7 +13129,7 @@
               <a:latin typeface="Aptos Narrow"/>
             </a:rPr>
             <a:pPr/>
-            <a:t>646</a:t>
+            <a:t>900</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="2000" b="1">
             <a:solidFill>
@@ -13536,7 +13365,7 @@
               <a:latin typeface="Aptos Narrow"/>
             </a:rPr>
             <a:pPr/>
-            <a:t>5</a:t>
+            <a:t>8</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="2000" b="1">
             <a:solidFill>
@@ -13772,7 +13601,7 @@
               <a:latin typeface="Aptos Narrow"/>
             </a:rPr>
             <a:pPr/>
-            <a:t>1140</a:t>
+            <a:t>2100</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="2000" b="1">
             <a:solidFill>
@@ -14045,7 +13874,7 @@
               <a:latin typeface="Aptos Narrow"/>
             </a:rPr>
             <a:pPr/>
-            <a:t>190</a:t>
+            <a:t>300</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="2000" b="1">
             <a:solidFill>
@@ -15124,7 +14953,7 @@
                 <a:latin typeface="Aptos Narrow"/>
               </a:rPr>
               <a:pPr/>
-              <a:t>3230</a:t>
+              <a:t>7200</a:t>
             </a:fld>
             <a:endParaRPr lang="en-US" sz="2000" b="1">
               <a:solidFill>
@@ -15361,7 +15190,7 @@
               <a:latin typeface="Aptos Narrow"/>
             </a:rPr>
             <a:pPr/>
-            <a:t>646</a:t>
+            <a:t>900</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="2000" b="1">
             <a:solidFill>
@@ -15597,7 +15426,7 @@
               <a:latin typeface="Aptos Narrow"/>
             </a:rPr>
             <a:pPr/>
-            <a:t>5</a:t>
+            <a:t>8</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="2000" b="1">
             <a:solidFill>
@@ -15833,7 +15662,7 @@
               <a:latin typeface="Aptos Narrow"/>
             </a:rPr>
             <a:pPr/>
-            <a:t>1140</a:t>
+            <a:t>2100</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="2000" b="1">
             <a:solidFill>
@@ -16106,7 +15935,7 @@
               <a:latin typeface="Aptos Narrow"/>
             </a:rPr>
             <a:pPr/>
-            <a:t>190</a:t>
+            <a:t>300</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="2000" b="1">
             <a:solidFill>
@@ -16610,6 +16439,56 @@
         <a:xfrm>
           <a:off x="9578340" y="220980"/>
           <a:ext cx="381000" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>449580</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>266700</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic macro="[0]!ExitFullScreen">
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Graphic 11" descr="Back with solid fill">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{40692CFF-E048-4B63-AA27-5514EA00B3D1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId19"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8983980" y="198120"/>
+          <a:ext cx="426720" cy="426720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -17953,13 +17832,13 @@
       <items count="10">
         <item h="1" x="8"/>
         <item h="1" x="6"/>
-        <item x="7"/>
+        <item h="1" x="7"/>
         <item h="1" x="3"/>
         <item h="1" x="5"/>
         <item h="1" x="0"/>
         <item h="1" x="2"/>
         <item h="1" x="1"/>
-        <item h="1" x="4"/>
+        <item x="4"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -18364,13 +18243,13 @@
   </rowFields>
   <rowItems count="4">
     <i>
-      <x v="1"/>
+      <x/>
+    </i>
+    <i>
+      <x v="3"/>
     </i>
     <i>
       <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -18416,12 +18295,12 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="2">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="1223" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="1349" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
             <customFilter operator="greaterThanOrEqual" val="44927"/>
-            <customFilter operator="lessThanOrEqual" val="45107"/>
+            <customFilter operator="lessThanOrEqual" val="44985"/>
           </customFilters>
         </filterColumn>
       </autoFilter>
@@ -18452,7 +18331,7 @@
 
 <file path=xl/pivotTables/pivotTable11.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{81106AAC-D9B2-4FC1-9230-462032F2416C}" name="PivotTable6" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="products by total amount">
-  <location ref="A35:B39" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A35:B37" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
     <pivotField numFmtId="14" showAll="0">
@@ -18503,17 +18382,17 @@
     </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0" measureFilter="1" sortType="descending">
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
       <items count="10">
         <item x="4"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item x="5"/>
-        <item x="3"/>
-        <item x="7"/>
-        <item x="6"/>
-        <item x="8"/>
+        <item h="1" x="1"/>
+        <item h="1" x="2"/>
+        <item h="1" x="0"/>
+        <item h="1" x="5"/>
+        <item h="1" x="3"/>
+        <item h="1" x="7"/>
+        <item h="1" x="6"/>
+        <item h="1" x="8"/>
         <item t="default"/>
       </items>
       <autoSortScope>
@@ -18925,15 +18804,9 @@
   <rowFields count="1">
     <field x="4"/>
   </rowFields>
-  <rowItems count="4">
+  <rowItems count="2">
     <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="4"/>
+      <x/>
     </i>
     <i t="grand">
       <x/>
@@ -18975,13 +18848,13 @@
     </chartFormat>
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <filters count="2">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="1225" name="Date">
+  <filters count="1">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="1351" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
             <customFilter operator="greaterThanOrEqual" val="44927"/>
-            <customFilter operator="lessThanOrEqual" val="45107"/>
+            <customFilter operator="lessThanOrEqual" val="44985"/>
           </customFilters>
         </filterColumn>
       </autoFilter>
@@ -18990,13 +18863,6 @@
           <x15:pivotFilter useWholeDay="1"/>
         </ext>
       </extLst>
-    </filter>
-    <filter fld="4" type="count" evalOrder="-1" id="777" iMeasureFld="0">
-      <autoFilter ref="A1">
-        <filterColumn colId="0">
-          <top10 val="3" filterVal="3"/>
-        </filterColumn>
-      </autoFilter>
     </filter>
   </filters>
   <extLst>
@@ -19067,13 +18933,13 @@
       <items count="10">
         <item h="1" x="8"/>
         <item h="1" x="6"/>
-        <item x="7"/>
+        <item h="1" x="7"/>
         <item h="1" x="3"/>
         <item h="1" x="5"/>
         <item h="1" x="0"/>
         <item h="1" x="2"/>
         <item h="1" x="1"/>
-        <item h="1" x="4"/>
+        <item x="4"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -19484,12 +19350,12 @@
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="1222" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="1348" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
             <customFilter operator="greaterThanOrEqual" val="44927"/>
-            <customFilter operator="lessThanOrEqual" val="45107"/>
+            <customFilter operator="lessThanOrEqual" val="44985"/>
           </customFilters>
         </filterColumn>
       </autoFilter>
@@ -19513,7 +19379,7 @@
 
 <file path=xl/pivotTables/pivotTable13.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F2128458-EC56-4BEB-8955-C6F5088054A7}" name="PivotTable4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="saleman by total amount">
-  <location ref="D20:E25" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="D20:E26" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
     <pivotField numFmtId="14" showAll="0">
@@ -19579,13 +19445,13 @@
       <items count="10">
         <item h="1" x="8"/>
         <item h="1" x="6"/>
-        <item x="7"/>
+        <item h="1" x="7"/>
         <item h="1" x="3"/>
         <item h="1" x="5"/>
         <item h="1" x="0"/>
         <item h="1" x="2"/>
         <item h="1" x="1"/>
-        <item h="1" x="4"/>
+        <item x="4"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -19988,12 +19854,15 @@
   <rowFields count="1">
     <field x="2"/>
   </rowFields>
-  <rowItems count="5">
+  <rowItems count="6">
     <i>
       <x/>
     </i>
     <i>
       <x v="1"/>
+    </i>
+    <i>
+      <x v="3"/>
     </i>
     <i>
       <x v="4"/>
@@ -20013,12 +19882,12 @@
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="1222" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="1348" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
             <customFilter operator="greaterThanOrEqual" val="44927"/>
-            <customFilter operator="lessThanOrEqual" val="45107"/>
+            <customFilter operator="lessThanOrEqual" val="44985"/>
           </customFilters>
         </filterColumn>
       </autoFilter>
@@ -20042,7 +19911,7 @@
 
 <file path=xl/pivotTables/pivotTable14.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{615A7D4C-F3B0-4140-8474-8DC713A1D055}" name="PivotTable3" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="saleman by total amount">
-  <location ref="D4:E9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="D4:E10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
     <pivotField numFmtId="14" showAll="0">
@@ -20108,13 +19977,13 @@
       <items count="10">
         <item h="1" x="8"/>
         <item h="1" x="6"/>
-        <item x="7"/>
+        <item h="1" x="7"/>
         <item h="1" x="3"/>
         <item h="1" x="5"/>
         <item h="1" x="0"/>
         <item h="1" x="2"/>
         <item h="1" x="1"/>
-        <item h="1" x="4"/>
+        <item x="4"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -20517,12 +20386,15 @@
   <rowFields count="1">
     <field x="2"/>
   </rowFields>
-  <rowItems count="5">
+  <rowItems count="6">
     <i>
       <x/>
     </i>
     <i>
       <x v="1"/>
+    </i>
+    <i>
+      <x v="3"/>
     </i>
     <i>
       <x v="4"/>
@@ -20553,12 +20425,12 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="1222" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="1348" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
             <customFilter operator="greaterThanOrEqual" val="44927"/>
-            <customFilter operator="lessThanOrEqual" val="45107"/>
+            <customFilter operator="lessThanOrEqual" val="44985"/>
           </customFilters>
         </filterColumn>
       </autoFilter>
@@ -20636,13 +20508,13 @@
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
         <item h="1" x="6"/>
-        <item x="7"/>
+        <item h="1" x="7"/>
         <item h="1" x="3"/>
         <item h="1" x="5"/>
         <item h="1" x="0"/>
         <item h="1" x="2"/>
         <item h="1" x="1"/>
-        <item h="1" x="4"/>
+        <item x="4"/>
         <item h="1" x="8"/>
         <item t="default"/>
       </items>
@@ -21048,7 +20920,7 @@
   </rowFields>
   <rowItems count="2">
     <i>
-      <x v="1"/>
+      <x v="7"/>
     </i>
     <i t="grand">
       <x/>
@@ -21062,12 +20934,12 @@
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="1222" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="1348" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
             <customFilter operator="greaterThanOrEqual" val="44927"/>
-            <customFilter operator="lessThanOrEqual" val="45107"/>
+            <customFilter operator="lessThanOrEqual" val="44985"/>
           </customFilters>
         </filterColumn>
       </autoFilter>
@@ -21091,7 +20963,7 @@
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2A05D2F9-2E80-4787-913B-C1FC915A823D}" name="PivotTable13" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9" rowHeaderCaption="products by total amount">
-  <location ref="H4:I7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="H4:I6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
     <pivotField numFmtId="14" showAll="0">
@@ -21146,13 +21018,13 @@
       <items count="10">
         <item h="1" x="8"/>
         <item h="1" x="6"/>
-        <item x="7"/>
+        <item h="1" x="7"/>
         <item h="1" x="3"/>
         <item h="1" x="5"/>
         <item h="1" x="0"/>
         <item h="1" x="2"/>
         <item h="1" x="1"/>
-        <item h="1" x="4"/>
+        <item x="4"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -21555,12 +21427,9 @@
   <rowFields count="1">
     <field x="9"/>
   </rowFields>
-  <rowItems count="3">
+  <rowItems count="2">
     <i>
       <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
     </i>
     <i t="grand">
       <x/>
@@ -21603,12 +21472,12 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="1222" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="1348" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
             <customFilter operator="greaterThanOrEqual" val="44927"/>
-            <customFilter operator="lessThanOrEqual" val="45107"/>
+            <customFilter operator="lessThanOrEqual" val="44985"/>
           </customFilters>
         </filterColumn>
       </autoFilter>
@@ -21687,13 +21556,13 @@
       <items count="10">
         <item h="1" x="8"/>
         <item h="1" x="6"/>
-        <item x="7"/>
+        <item h="1" x="7"/>
         <item h="1" x="3"/>
         <item h="1" x="5"/>
         <item h="1" x="0"/>
         <item h="1" x="2"/>
         <item h="1" x="1"/>
-        <item h="1" x="4"/>
+        <item x="4"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -22104,12 +21973,12 @@
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="1222" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="1348" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
             <customFilter operator="greaterThanOrEqual" val="44927"/>
-            <customFilter operator="lessThanOrEqual" val="45107"/>
+            <customFilter operator="lessThanOrEqual" val="44985"/>
           </customFilters>
         </filterColumn>
       </autoFilter>
@@ -22188,13 +22057,13 @@
       <items count="10">
         <item h="1" x="8"/>
         <item h="1" x="6"/>
-        <item x="7"/>
+        <item h="1" x="7"/>
         <item h="1" x="3"/>
         <item h="1" x="5"/>
         <item h="1" x="0"/>
         <item h="1" x="2"/>
         <item h="1" x="1"/>
-        <item h="1" x="4"/>
+        <item x="4"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -22605,12 +22474,12 @@
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="1222" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="1348" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
             <customFilter operator="greaterThanOrEqual" val="44927"/>
-            <customFilter operator="lessThanOrEqual" val="45107"/>
+            <customFilter operator="lessThanOrEqual" val="44985"/>
           </customFilters>
         </filterColumn>
       </autoFilter>
@@ -22689,13 +22558,13 @@
       <items count="10">
         <item h="1" x="8"/>
         <item h="1" x="6"/>
-        <item x="7"/>
+        <item h="1" x="7"/>
         <item h="1" x="3"/>
         <item h="1" x="5"/>
         <item h="1" x="0"/>
         <item h="1" x="2"/>
         <item h="1" x="1"/>
-        <item h="1" x="4"/>
+        <item x="4"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -23106,12 +22975,12 @@
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="1222" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="1348" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
             <customFilter operator="greaterThanOrEqual" val="44927"/>
-            <customFilter operator="lessThanOrEqual" val="45107"/>
+            <customFilter operator="lessThanOrEqual" val="44985"/>
           </customFilters>
         </filterColumn>
       </autoFilter>
@@ -23189,13 +23058,13 @@
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
         <item h="1" x="6"/>
-        <item x="7"/>
+        <item h="1" x="7"/>
         <item h="1" x="3"/>
         <item h="1" x="5"/>
         <item h="1" x="0"/>
         <item h="1" x="2"/>
         <item h="1" x="1"/>
-        <item h="1" x="4"/>
+        <item x="4"/>
         <item h="1" x="8"/>
         <item t="default"/>
       </items>
@@ -23601,7 +23470,7 @@
   </rowFields>
   <rowItems count="2">
     <i>
-      <x v="1"/>
+      <x v="7"/>
     </i>
     <i t="grand">
       <x/>
@@ -23615,12 +23484,12 @@
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="1222" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="1348" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
             <customFilter operator="greaterThanOrEqual" val="44927"/>
-            <customFilter operator="lessThanOrEqual" val="45107"/>
+            <customFilter operator="lessThanOrEqual" val="44985"/>
           </customFilters>
         </filterColumn>
       </autoFilter>
@@ -23699,13 +23568,13 @@
       <items count="10">
         <item h="1" x="8"/>
         <item h="1" x="6"/>
-        <item x="7"/>
+        <item h="1" x="7"/>
         <item h="1" x="3"/>
         <item h="1" x="5"/>
         <item h="1" x="0"/>
         <item h="1" x="2"/>
         <item h="1" x="1"/>
-        <item h="1" x="4"/>
+        <item x="4"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -24116,12 +23985,12 @@
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="1222" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="1348" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
             <customFilter operator="greaterThanOrEqual" val="44927"/>
-            <customFilter operator="lessThanOrEqual" val="45107"/>
+            <customFilter operator="lessThanOrEqual" val="44985"/>
           </customFilters>
         </filterColumn>
       </autoFilter>
@@ -24145,7 +24014,7 @@
 
 <file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{03CCA7B5-97F8-4219-AD97-3CE5BBB7E6F2}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="13" rowHeaderCaption="products by total amount">
-  <location ref="A4:B14" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A4:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
     <pivotField numFmtId="14" showAll="0">
@@ -24198,15 +24067,15 @@
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item x="6"/>
-        <item x="7"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
+        <item h="1" x="6"/>
+        <item h="1" x="7"/>
+        <item h="1" x="3"/>
+        <item h="1" x="5"/>
+        <item h="1" x="0"/>
+        <item h="1" x="2"/>
+        <item h="1" x="1"/>
         <item x="4"/>
-        <item x="8"/>
+        <item h="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -24609,33 +24478,9 @@
   <rowFields count="1">
     <field x="4"/>
   </rowFields>
-  <rowItems count="10">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
+  <rowItems count="2">
     <i>
       <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
     </i>
     <i t="grand">
       <x/>
@@ -24687,12 +24532,12 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="1222" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="1348" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
             <customFilter operator="greaterThanOrEqual" val="44927"/>
-            <customFilter operator="lessThanOrEqual" val="45107"/>
+            <customFilter operator="lessThanOrEqual" val="44985"/>
           </customFilters>
         </filterColumn>
       </autoFilter>
@@ -24728,19 +24573,21 @@
     <pivotTable tabId="8" name="PivotTable9"/>
     <pivotTable tabId="8" name="PivotTable13"/>
     <pivotTable tabId="8" name="PivotTable14"/>
+    <pivotTable tabId="8" name="PivotTable2"/>
+    <pivotTable tabId="8" name="PivotTable6"/>
   </pivotTables>
   <data>
     <tabular pivotCacheId="2123660732">
       <items count="9">
         <i x="8"/>
         <i x="6"/>
-        <i x="7" s="1"/>
+        <i x="7"/>
         <i x="3"/>
         <i x="5"/>
         <i x="0"/>
         <i x="2"/>
         <i x="1"/>
-        <i x="4"/>
+        <i x="4" s="1"/>
       </items>
     </tabular>
   </data>
@@ -25178,7 +25025,7 @@
     <pivotTable tabId="8" name="PivotTable14"/>
   </pivotTables>
   <state minimalRefreshVersion="6" lastRefreshVersion="6" pivotCacheId="2123660732" filterType="dateBetween">
-    <selection startDate="2023-01-01T00:00:00" endDate="2023-06-30T00:00:00"/>
+    <selection startDate="2023-01-01T00:00:00" endDate="2023-02-28T00:00:00"/>
     <bounds startDate="2023-01-01T00:00:00" endDate="2024-01-01T00:00:00"/>
   </state>
 </timelineCacheDefinition>
@@ -25186,19 +25033,19 @@
 
 <file path=xl/timelines/timeline1.xml><?xml version="1.0" encoding="utf-8"?>
 <timelines xmlns="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <timeline name="Date 2" xr10:uid="{47AEEC7F-1B59-42CD-AC3E-005E93700E69}" cache="NativeTimeline_Date" caption="Date" showHeader="0" showSelectionLabel="0" showTimeLevel="0" showHorizontalScrollbar="0" level="2" selectionLevel="1" scrollPosition="2023-01-01T00:00:00" style="lala"/>
+  <timeline name="Date 2" xr10:uid="{47AEEC7F-1B59-42CD-AC3E-005E93700E69}" cache="NativeTimeline_Date" caption="Date" showHeader="0" showSelectionLabel="0" showTimeLevel="0" showHorizontalScrollbar="0" level="2" selectionLevel="2" scrollPosition="2023-01-01T00:00:00" style="lala"/>
 </timelines>
 </file>
 
 <file path=xl/timelines/timeline2.xml><?xml version="1.0" encoding="utf-8"?>
 <timelines xmlns="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <timeline name="Date 3" xr10:uid="{CE1DB49B-9349-487E-9E64-4BEE34AC5625}" cache="NativeTimeline_Date" caption="Date" showHeader="0" showSelectionLabel="0" showTimeLevel="0" showHorizontalScrollbar="0" level="2" selectionLevel="1" scrollPosition="2023-01-01T00:00:00" style="lala"/>
+  <timeline name="Date 3" xr10:uid="{CE1DB49B-9349-487E-9E64-4BEE34AC5625}" cache="NativeTimeline_Date" caption="Date" showHeader="0" showSelectionLabel="0" showTimeLevel="0" showHorizontalScrollbar="0" level="2" selectionLevel="2" scrollPosition="2023-01-01T00:00:00" style="lala"/>
 </timelines>
 </file>
 
 <file path=xl/timelines/timeline3.xml><?xml version="1.0" encoding="utf-8"?>
 <timelines xmlns="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <timeline name="Date 1" xr10:uid="{85528314-E4CD-4A7C-82A1-1078B90ECD66}" cache="NativeTimeline_Date" caption="Date" showHeader="0" showSelectionLabel="0" showTimeLevel="0" showHorizontalScrollbar="0" level="2" selectionLevel="1" scrollPosition="2023-01-01T00:00:00" style="lala"/>
+  <timeline name="Date 1" xr10:uid="{85528314-E4CD-4A7C-82A1-1078B90ECD66}" cache="NativeTimeline_Date" caption="Date" showHeader="0" showSelectionLabel="0" showTimeLevel="0" showHorizontalScrollbar="0" level="2" selectionLevel="2" scrollPosition="2023-01-01T00:00:00" style="lala"/>
 </timelines>
 </file>
 
@@ -25295,7 +25142,7 @@
   <dimension ref="A1:O58"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.5546875" bestFit="1" customWidth="1"/>
@@ -25343,142 +25190,90 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B5" s="12">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>50</v>
       </c>
       <c r="E5" s="12">
-        <v>1140</v>
+        <v>900</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>79</v>
       </c>
       <c r="I5" s="12">
-        <v>2850</v>
+        <v>7200</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>67</v>
+        <v>14</v>
       </c>
       <c r="B6" s="12">
-        <v>3230</v>
+        <v>7200</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>53</v>
       </c>
       <c r="E6" s="12">
-        <v>760</v>
+        <v>2400</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>80</v>
+        <v>14</v>
       </c>
       <c r="I6" s="12">
-        <v>380</v>
+        <v>7200</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="B7" s="12">
-        <v>306000</v>
-      </c>
       <c r="D7" s="11" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E7" s="12">
-        <v>1140</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="I7" s="12">
-        <v>3230</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="B8" s="12">
-        <v>12000</v>
-      </c>
       <c r="D8" s="11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E8" s="12">
-        <v>190</v>
+        <v>300</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="B9" s="12">
-        <v>4200</v>
-      </c>
       <c r="D9" s="11" t="s">
-        <v>14</v>
+        <v>59</v>
       </c>
       <c r="E9" s="12">
-        <v>3230</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="B10" s="12">
-        <v>79800</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="B11" s="12">
-        <v>10500</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="B12" s="12">
+      <c r="D10" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="12">
         <v>7200</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="B13" s="12">
-        <v>168</v>
-      </c>
       <c r="H13" s="10" t="s">
         <v>70</v>
       </c>
       <c r="I13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" s="12">
-        <v>426698</v>
-      </c>
       <c r="H14" s="11" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="I14" s="12">
-        <v>190</v>
+        <v>300</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
@@ -25486,7 +25281,7 @@
         <v>14</v>
       </c>
       <c r="I15" s="12">
-        <v>190</v>
+        <v>300</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
@@ -25499,10 +25294,10 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B19" s="12">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
@@ -25510,7 +25305,7 @@
         <v>14</v>
       </c>
       <c r="B20" s="12">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>69</v>
@@ -25524,7 +25319,7 @@
         <v>50</v>
       </c>
       <c r="E21" s="12">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
@@ -25532,12 +25327,12 @@
         <v>53</v>
       </c>
       <c r="E22" s="12">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D23" s="11" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E23" s="12">
         <v>2</v>
@@ -25545,7 +25340,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D24" s="11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E24" s="12">
         <v>1</v>
@@ -25553,10 +25348,18 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D25" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="E25" s="12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D26" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E25" s="12">
-        <v>5</v>
+      <c r="E26" s="12">
+        <v>8</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
@@ -25575,58 +25378,46 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B36" s="12">
-        <v>306000</v>
+        <v>7200</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E36" s="12">
-        <v>1140</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="B37" s="12">
-        <v>79800</v>
+        <v>7200</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="E37" s="12">
-        <v>760</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A38" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="B38" s="12">
-        <v>12000</v>
-      </c>
       <c r="D38" s="11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E38" s="12">
-        <v>1140</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A39" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B39" s="12">
-        <v>397800</v>
-      </c>
       <c r="D39" s="11" t="s">
         <v>14</v>
       </c>
       <c r="E39" s="12">
-        <v>3040</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
@@ -25716,39 +25507,39 @@
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A58" s="12">
-        <v>3230</v>
+        <v>7200</v>
       </c>
       <c r="B58" s="20">
         <f>GETPIVOTDATA("Amount",$A$57)</f>
-        <v>3230</v>
+        <v>7200</v>
       </c>
       <c r="D58" s="12">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E58" s="20">
         <f>GETPIVOTDATA("Amount",$D$57)</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H58" s="12">
-        <v>646</v>
+        <v>900</v>
       </c>
       <c r="I58" s="20">
         <f>GETPIVOTDATA("Amount",$H$57)</f>
-        <v>646</v>
+        <v>900</v>
       </c>
       <c r="K58" s="12">
-        <v>1140</v>
+        <v>2100</v>
       </c>
       <c r="L58" s="20">
         <f>GETPIVOTDATA("Amount",$K$57)</f>
-        <v>1140</v>
+        <v>2100</v>
       </c>
       <c r="N58" s="12">
-        <v>190</v>
+        <v>300</v>
       </c>
       <c r="O58" s="20">
         <f>GETPIVOTDATA("Amount",$N$57)</f>
-        <v>190</v>
+        <v>300</v>
       </c>
     </row>
   </sheetData>
@@ -26848,13 +26639,13 @@
         <v>45004</v>
       </c>
       <c r="C42" t="s">
+        <v>80</v>
+      </c>
+      <c r="D42" t="s">
         <v>81</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>82</v>
-      </c>
-      <c r="E42" t="s">
-        <v>83</v>
       </c>
       <c r="F42">
         <v>3</v>

</xml_diff>

<commit_message>
copy icons + coller in saleman and product sheet
</commit_message>
<xml_diff>
--- a/li.xlsx
+++ b/li.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\power bi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B005AF-28BA-4EC5-B32A-95197A5DA7F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EDC7306-B16E-45F0-BAEC-937C31437605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="705" activeTab="8" xr2:uid="{12120B74-1E2A-4740-BDBD-5E619114E9BB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="705" activeTab="6" xr2:uid="{12120B74-1E2A-4740-BDBD-5E619114E9BB}"/>
   </bookViews>
   <sheets>
     <sheet name="pivot table" sheetId="3" r:id="rId1"/>
@@ -12228,22 +12228,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>320040</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>144780</xdr:rowOff>
+      <xdr:colOff>220980</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>220980</xdr:colOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>601980</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>106680</xdr:rowOff>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
-    <xdr:pic>
+    <xdr:pic macro="[0]!FullScreen">
       <xdr:nvPicPr>
-        <xdr:cNvPr id="29" name="Graphic 28" descr="Arrow circle with solid fill">
+        <xdr:cNvPr id="28" name="Graphic 27" descr="Monitor with solid fill">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{68A5AFA2-93F0-63C0-127D-3C3C37C79AAF}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FC56FCBE-5CC0-46E3-B30A-7D7967C205E1}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -12265,8 +12265,58 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10683240" y="144780"/>
-          <a:ext cx="510540" cy="510540"/>
+          <a:off x="10584180" y="243840"/>
+          <a:ext cx="381000" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>236220</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>53340</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic macro="[0]!ExitFullScreen">
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="35" name="Graphic 34" descr="Back with solid fill">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{73917054-CA70-4266-891E-5ED2BA19435E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId19"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9989820" y="220980"/>
+          <a:ext cx="426720" cy="426720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -14334,6 +14384,106 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>327660</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>99060</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic macro="[0]!FullScreen">
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="28" name="Graphic 27" descr="Monitor with solid fill">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{630C1DA7-83CB-41B2-8138-A626748F2BBE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId17"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10081260" y="220980"/>
+          <a:ext cx="381000" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>160020</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic macro="[0]!ExitFullScreen">
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="29" name="Graphic 28" descr="Back with solid fill">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3F4BC3A5-1517-49CA-B2D2-EAC2FD45575A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId19"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9486900" y="198120"/>
+          <a:ext cx="426720" cy="426720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>

</xml_diff>